<commit_message>
Same Scanning and Many Processing Updates
</commit_message>
<xml_diff>
--- a/system_development/Orichalcum/v0.2/Software_design/v2-cover-control/VIBROMETER SCAN SETTINGS.xlsx
+++ b/system_development/Orichalcum/v0.2/Software_design/v2-cover-control/VIBROMETER SCAN SETTINGS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\In-situ-monitoring-of-powder-bed-fusion-additive-manufacturing\system_development\Orichalcum\v0.2\Software_design\v2-cover-control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80D26A8-021C-4F41-BFEE-7767015D84F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D063A036-9C91-402B-AA8B-3268F6780DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4980" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Parameters" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="141">
   <si>
     <t>Receiver</t>
   </si>
@@ -55,9 +55,6 @@
   </si>
   <si>
     <t>Trigger</t>
-  </si>
-  <si>
-    <t>Internal</t>
   </si>
   <si>
     <t>Pulse Amplitude</t>
@@ -238,9 +235,6 @@
     </r>
   </si>
   <si>
-    <t>Scan of…</t>
-  </si>
-  <si>
     <t xml:space="preserve">x count </t>
   </si>
   <si>
@@ -335,9 +329,6 @@
   </si>
   <si>
     <t>noisey/didn't run</t>
-  </si>
-  <si>
-    <t>20k</t>
   </si>
   <si>
     <t>Test Scan 6</t>
@@ -357,6 +348,133 @@
   <si>
     <t>Trigger
 Source</t>
+  </si>
+  <si>
+    <t>Channel 0,1</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>[1]</t>
+  </si>
+  <si>
+    <t>[2]</t>
+  </si>
+  <si>
+    <t>ECHO: sending and receiving pulse from same transducer; THROUGH: reading signal from another transducer</t>
+  </si>
+  <si>
+    <t>INT: Trigger from Pulser DPR300; EXT: Trigger from PXI (or external device)</t>
+  </si>
+  <si>
+    <t>INT</t>
+  </si>
+  <si>
+    <t>PULSER FOOTNOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Digitizer
+Channel</t>
+  </si>
+  <si>
+    <t>External Trig</t>
+  </si>
+  <si>
+    <t>Specimen</t>
+  </si>
+  <si>
+    <t>interal delay of 20us</t>
+  </si>
+  <si>
+    <t>DATA CHANNELS CORRECTED</t>
+  </si>
+  <si>
+    <t>Signal Scan 1</t>
+  </si>
+  <si>
+    <t>Channel 1</t>
+  </si>
+  <si>
+    <t>(data of interest: 'point-000-000-' in center)</t>
+  </si>
+  <si>
+    <t>35mm^2</t>
+  </si>
+  <si>
+    <t>20k</t>
+  </si>
+  <si>
+    <t>200k</t>
+  </si>
+  <si>
+    <t>Vibration Scan 1</t>
+  </si>
+  <si>
+    <t>Vibration Scan 2</t>
+  </si>
+  <si>
+    <t>Vibration Scan A</t>
+  </si>
+  <si>
+    <t>Vibration Scan B</t>
+  </si>
+  <si>
+    <t>point on welded surface</t>
+  </si>
+  <si>
+    <t>point on bare build plate</t>
+  </si>
+  <si>
+    <t>(4 square build plate)</t>
+  </si>
+  <si>
+    <t>Signal Scan 2</t>
+  </si>
+  <si>
+    <t>all squares on 4square plate</t>
+  </si>
+  <si>
+    <t>step</t>
+  </si>
+  <si>
+    <t>SS heatmap generated</t>
+  </si>
+  <si>
+    <t>center of build plate</t>
+  </si>
+  <si>
+    <t>Vibration Scan 3</t>
+  </si>
+  <si>
+    <t>first square</t>
+  </si>
+  <si>
+    <t>record length too short to catch meaningful waveforms</t>
+  </si>
+  <si>
+    <t>**</t>
+  </si>
+  <si>
+    <t>max freq = 2.25MHz</t>
+  </si>
+  <si>
+    <t>28mm^2</t>
+  </si>
+  <si>
+    <t>Vibration Scan 4</t>
+  </si>
+  <si>
+    <t>same as Row16 but with both channels</t>
+  </si>
+  <si>
+    <t>3D SS HTML &amp; 2D heatmap generated</t>
   </si>
 </sst>
 </file>
@@ -477,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -502,9 +620,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -536,10 +675,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,8 +702,8 @@
       <xdr:rowOff>41944</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>680438</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4147887</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>176028</xdr:rowOff>
     </xdr:to>
@@ -614,6 +749,50 @@
             </a14:hiddenFill>
           </a:ext>
         </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>15313</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>20972</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3854461</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>27963</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30FA26F3-D258-99C7-056F-70232EB75887}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7481515" y="3935834"/>
+          <a:ext cx="5370139" cy="4509083"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -819,274 +998,663 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F5A5D31-C167-4FC4-94A5-027E9DD85F49}">
-  <dimension ref="B2:O10"/>
+  <dimension ref="B2:P19"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.21875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
-    <col min="4" max="5" width="10.21875" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8" customWidth="1"/>
-    <col min="9" max="11" width="8.109375" customWidth="1"/>
-    <col min="13" max="13" width="9.6640625" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" customWidth="1"/>
+    <col min="7" max="7" width="7.88671875" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" customWidth="1"/>
+    <col min="10" max="12" width="8.109375" customWidth="1"/>
+    <col min="13" max="13" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.6640625" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="11" t="s">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B3"/>
+    </row>
+    <row r="4" spans="2:16" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B4" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="6"/>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3"/>
-    </row>
-    <row r="4" spans="2:15" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="B4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="9" t="s">
+      <c r="J4" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H4" s="10" t="s">
+      <c r="K4" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="L4" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="K4" s="10" t="s">
+      <c r="M4" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="P4" s="16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="C5" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M4" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="H5">
-        <v>50</v>
-      </c>
+      <c r="H5" s="6"/>
       <c r="I5">
         <v>50</v>
       </c>
       <c r="J5">
+        <v>50</v>
+      </c>
+      <c r="K5">
         <v>-700</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>500</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>14</v>
       </c>
-      <c r="N5" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O5" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="G6" s="6"/>
-      <c r="H6">
-        <v>60</v>
-      </c>
+      <c r="H6" s="6"/>
       <c r="I6">
         <v>60</v>
       </c>
       <c r="J6">
+        <v>60</v>
+      </c>
+      <c r="K6">
         <v>-900</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>200</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>15</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="O6" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="5" t="s">
-        <v>86</v>
-      </c>
       <c r="C7" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="G7" s="6"/>
-      <c r="H7">
-        <v>50</v>
-      </c>
+      <c r="H7" s="6"/>
       <c r="I7">
         <v>50</v>
       </c>
       <c r="J7">
+        <v>50</v>
+      </c>
+      <c r="K7">
         <v>-1000</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>0</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>20</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="O7" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="P7" t="s">
         <v>85</v>
       </c>
-      <c r="O7" t="s">
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6">
+        <v>50</v>
+      </c>
+      <c r="J8">
+        <v>50</v>
+      </c>
+      <c r="K8">
+        <v>-700</v>
+      </c>
+      <c r="L8">
+        <v>300</v>
+      </c>
+      <c r="M8">
+        <v>14</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>50</v>
-      </c>
-      <c r="J8">
-        <v>-700</v>
-      </c>
-      <c r="K8">
-        <v>300</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6">
+        <v>25</v>
+      </c>
+      <c r="J9">
+        <v>25</v>
+      </c>
+      <c r="K9">
+        <v>-380</v>
+      </c>
+      <c r="L9">
+        <v>600</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
+      <c r="N9">
+        <v>32</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="G9" s="6">
-        <v>10000</v>
-      </c>
-      <c r="H9" s="6">
+      <c r="P9" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="I10" s="6">
         <v>25</v>
       </c>
-      <c r="I9">
+      <c r="J10">
         <v>25</v>
       </c>
-      <c r="J9">
+      <c r="K10">
         <v>-380</v>
       </c>
-      <c r="K9">
+      <c r="L10">
         <v>600</v>
       </c>
-      <c r="L9">
+      <c r="M10">
         <v>10</v>
       </c>
-      <c r="M9">
+      <c r="N10">
         <v>32</v>
       </c>
-      <c r="N9" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="O10" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>70</v>
+      <c r="P10" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P11" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="I12" s="6">
+        <v>25</v>
+      </c>
+      <c r="J12">
+        <v>25</v>
+      </c>
+      <c r="K12">
+        <v>-380</v>
+      </c>
+      <c r="L12">
+        <v>600</v>
+      </c>
+      <c r="M12">
+        <v>10</v>
+      </c>
+      <c r="N12">
+        <v>32</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I13" s="6">
+        <v>20</v>
+      </c>
+      <c r="J13">
+        <v>20</v>
+      </c>
+      <c r="K13">
+        <v>-360</v>
+      </c>
+      <c r="L13">
+        <v>630</v>
+      </c>
+      <c r="M13">
+        <v>10</v>
+      </c>
+      <c r="N13">
+        <v>32</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="6">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>-280</v>
+      </c>
+      <c r="L14">
+        <v>690</v>
+      </c>
+      <c r="N14">
+        <v>32</v>
+      </c>
+      <c r="O14" s="6"/>
+      <c r="P14" s="18" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="6">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>-280</v>
+      </c>
+      <c r="L15">
+        <v>720</v>
+      </c>
+      <c r="N15">
+        <v>32</v>
+      </c>
+      <c r="P15" s="18"/>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="I16" s="6">
+        <v>25</v>
+      </c>
+      <c r="J16">
+        <v>25</v>
+      </c>
+      <c r="K16">
+        <v>-340</v>
+      </c>
+      <c r="L16">
+        <v>630</v>
+      </c>
+      <c r="M16">
+        <v>8</v>
+      </c>
+      <c r="O16" t="s">
+        <v>137</v>
+      </c>
+      <c r="P16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="6">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>-280</v>
+      </c>
+      <c r="L17">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="I18" s="6">
+        <v>15</v>
+      </c>
+      <c r="J18">
+        <v>15</v>
+      </c>
+      <c r="K18">
+        <v>-235</v>
+      </c>
+      <c r="L18">
+        <v>630</v>
+      </c>
+      <c r="M18">
+        <v>6</v>
+      </c>
+      <c r="P18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I19" s="6">
+        <v>25</v>
+      </c>
+      <c r="J19">
+        <v>25</v>
+      </c>
+      <c r="K19">
+        <v>-340</v>
+      </c>
+      <c r="L19">
+        <v>630</v>
+      </c>
+      <c r="M19">
+        <v>8</v>
+      </c>
+      <c r="N19">
+        <v>64</v>
+      </c>
+      <c r="O19" t="s">
+        <v>137</v>
+      </c>
+      <c r="P19" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="P14:P15"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1099,7 +1667,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:I1001"/>
+  <dimension ref="B1:L1001"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.33203125" customWidth="1"/>
@@ -1111,36 +1679,46 @@
     <col min="8" max="8" width="6.21875" style="3" customWidth="1"/>
     <col min="9" max="9" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="12" max="12" width="94.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C2" s="20" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="28"/>
+      <c r="E2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="21"/>
-      <c r="F2" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="G2" s="26"/>
+      <c r="H2" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="E3" t="s">
+        <v>102</v>
+      </c>
       <c r="F3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1148,13 +1726,13 @@
         <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1162,13 +1740,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1176,15 +1754,15 @@
         <v>5</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="1" t="s">
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>5</v>
@@ -1194,119 +1772,125 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="26"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="19"/>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C9" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="D9" s="1">
         <v>16</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="4" t="s">
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="G10" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C11" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G11" s="3">
         <v>200000</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" s="21"/>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="28"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C14" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C15" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15" s="3">
         <v>5</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H15" s="3">
         <v>0.8</v>
       </c>
       <c r="I15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C16" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" s="3">
         <v>1</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="I16" s="17"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I16" s="24"/>
+      <c r="K16" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C17" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G17" s="6">
         <v>0</v>
@@ -1314,75 +1898,99 @@
       <c r="H17" s="3">
         <v>90</v>
       </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="K17" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="L17" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C18" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G18">
-        <f>-(H18-H$17)*(H$15)*(100)</f>
+        <f t="shared" ref="G18:G23" si="0">-(H18-H$17)*(H$15)*(100)</f>
         <v>80</v>
       </c>
       <c r="H18" s="3">
         <v>89</v>
       </c>
       <c r="I18" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="L18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="F19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G19">
-        <f t="shared" ref="G19:G23" si="0">-(H19-H$17)*(H$15)*(100)</f>
+        <f t="shared" si="0"/>
         <v>160</v>
       </c>
       <c r="H19" s="3">
         <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="L19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C20" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" s="3">
         <v>200000</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G20">
-        <f>-(H20-H$17)*(H$15)*(100)</f>
+        <f t="shared" si="0"/>
         <v>240.00000000000003</v>
       </c>
       <c r="H20" s="3">
         <v>87</v>
       </c>
       <c r="I20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="L20" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C21" s="1"/>
       <c r="D21" s="3"/>
       <c r="F21" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G21">
         <f t="shared" si="0"/>
@@ -1392,21 +2000,21 @@
         <v>86</v>
       </c>
       <c r="I21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="20" t="s">
         <v>6</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G22">
         <f t="shared" si="0"/>
@@ -1416,19 +2024,19 @@
         <v>85</v>
       </c>
       <c r="I22" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="20"/>
       <c r="C23" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D23" s="3">
         <v>-0.2</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G23">
         <f t="shared" si="0"/>
@@ -1438,143 +2046,146 @@
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="13"/>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="20"/>
       <c r="C24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="20"/>
+      <c r="C25" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D25" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="13"/>
-      <c r="C25" s="4" t="s">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="20"/>
+      <c r="C26" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="13"/>
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C27" s="1"/>
       <c r="D27" s="3"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C28" s="1"/>
       <c r="D28" s="3"/>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D29" s="12"/>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C29" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="19"/>
       <c r="F29" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C30" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D30" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C31" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D31" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C32" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C33" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C34" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C33" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C34" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="D34" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C35" s="1"/>
-    </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C36" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D36" s="12"/>
-    </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="L35" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C36" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36" s="19"/>
+    </row>
+    <row r="37" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C37" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C38" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C39" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C40" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C41" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C40" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C41" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C42" s="1"/>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C43" s="1"/>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C44" s="1"/>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C45" s="1"/>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C46" s="1"/>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C47" s="1"/>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C48" s="1"/>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>